<commit_message>
update ground truth analysis, and old new comparison analysis
</commit_message>
<xml_diff>
--- a/ground truth analysis/Ground-Truth-150 Dec 5.xlsx
+++ b/ground truth analysis/Ground-Truth-150 Dec 5.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaimingtao/Library/CloudStorage/Dropbox/Shared/ChatGPT/FineTuningPaper/PLOSOne/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaimingtao/HIVDB/chat_HIVDB_paper/ground truth analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D3019A-4570-CA48-AFAE-135528D1B7E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F868E3F7-CFDA-AE48-8462-E8E2B6978823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12020" yWindow="500" windowWidth="37460" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="940" yWindow="500" windowWidth="37460" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -656,9 +656,6 @@
     <t>Sanger</t>
   </si>
   <si>
-    <t>Human-Answer corrected</t>
-  </si>
-  <si>
     <t>MW484894, MW484895, MW484893, DQ380549, AF492618, MW48492</t>
   </si>
   <si>
@@ -972,6 +969,9 @@
   </si>
   <si>
     <t>Not known</t>
+  </si>
+  <si>
+    <t>Human-Answer</t>
   </si>
 </sst>
 </file>
@@ -1443,7 +1443,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>206</v>
+        <v>311</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -6963,7 +6963,7 @@
         <v>7</v>
       </c>
       <c r="F277" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="278" spans="1:6" x14ac:dyDescent="0.2">
@@ -7843,7 +7843,7 @@
         <v>31</v>
       </c>
       <c r="F321" s="10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.2">
@@ -9123,7 +9123,7 @@
         <v>31</v>
       </c>
       <c r="F385" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="386" spans="1:6" x14ac:dyDescent="0.2">
@@ -11363,7 +11363,7 @@
         <v>31</v>
       </c>
       <c r="F497" s="10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="498" spans="1:6" x14ac:dyDescent="0.2">
@@ -16263,7 +16263,7 @@
         <v>7</v>
       </c>
       <c r="F742" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="743" spans="1:6" x14ac:dyDescent="0.2">
@@ -18543,7 +18543,7 @@
         <v>18</v>
       </c>
       <c r="F856" s="10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="857" spans="1:6" x14ac:dyDescent="0.2">
@@ -18903,7 +18903,7 @@
         <v>22</v>
       </c>
       <c r="F874" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="875" spans="1:6" x14ac:dyDescent="0.2">
@@ -19143,7 +19143,7 @@
         <v>7</v>
       </c>
       <c r="F886" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="887" spans="1:6" x14ac:dyDescent="0.2">
@@ -19223,7 +19223,7 @@
         <v>22</v>
       </c>
       <c r="F890" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="891" spans="1:6" x14ac:dyDescent="0.2">
@@ -20223,7 +20223,7 @@
         <v>22</v>
       </c>
       <c r="F940" s="10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="941" spans="1:6" x14ac:dyDescent="0.2">
@@ -24983,7 +24983,7 @@
         <v>22</v>
       </c>
       <c r="F1178" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="1179" spans="1:6" x14ac:dyDescent="0.2">
@@ -27463,7 +27463,7 @@
         <v>7</v>
       </c>
       <c r="F1302" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="1303" spans="1:6" x14ac:dyDescent="0.2">
@@ -28443,7 +28443,7 @@
         <v>18</v>
       </c>
       <c r="F1351" s="10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="1352" spans="1:6" x14ac:dyDescent="0.2">
@@ -29143,7 +29143,7 @@
         <v>22</v>
       </c>
       <c r="F1386" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="1387" spans="1:6" x14ac:dyDescent="0.2">
@@ -30663,7 +30663,7 @@
         <v>7</v>
       </c>
       <c r="F1462" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="1463" spans="1:6" x14ac:dyDescent="0.2">
@@ -31943,7 +31943,7 @@
         <v>7</v>
       </c>
       <c r="F1526" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="1527" spans="1:6" x14ac:dyDescent="0.2">
@@ -36463,7 +36463,7 @@
         <v>18</v>
       </c>
       <c r="F1752" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="1753" spans="1:6" x14ac:dyDescent="0.2">
@@ -37503,7 +37503,7 @@
         <v>22</v>
       </c>
       <c r="F1804" s="10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="1805" spans="1:6" x14ac:dyDescent="0.2">
@@ -39923,7 +39923,7 @@
         <v>7</v>
       </c>
       <c r="F1925" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="1926" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -39963,7 +39963,7 @@
         <v>18</v>
       </c>
       <c r="F1927" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="1928" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -39983,7 +39983,7 @@
         <v>18</v>
       </c>
       <c r="F1928" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1929" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40163,7 +40163,7 @@
         <v>31</v>
       </c>
       <c r="F1937" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="1938" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40243,7 +40243,7 @@
         <v>7</v>
       </c>
       <c r="F1941" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="1942" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40283,7 +40283,7 @@
         <v>18</v>
       </c>
       <c r="F1943" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="1944" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40343,7 +40343,7 @@
         <v>22</v>
       </c>
       <c r="F1946" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="1947" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -40363,7 +40363,7 @@
         <v>22</v>
       </c>
       <c r="F1947" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="1948" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40403,7 +40403,7 @@
         <v>31</v>
       </c>
       <c r="F1949" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="1950" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -40563,7 +40563,7 @@
         <v>7</v>
       </c>
       <c r="F1957" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="1958" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40623,7 +40623,7 @@
         <v>18</v>
       </c>
       <c r="F1960" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="1961" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40663,7 +40663,7 @@
         <v>22</v>
       </c>
       <c r="F1962" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="1963" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -40803,7 +40803,7 @@
         <v>31</v>
       </c>
       <c r="F1969" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="1970" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40883,7 +40883,7 @@
         <v>7</v>
       </c>
       <c r="F1973" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="1974" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40923,7 +40923,7 @@
         <v>18</v>
       </c>
       <c r="F1975" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="1976" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40943,7 +40943,7 @@
         <v>18</v>
       </c>
       <c r="F1976" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="1977" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -40983,7 +40983,7 @@
         <v>22</v>
       </c>
       <c r="F1978" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="1979" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -41003,7 +41003,7 @@
         <v>22</v>
       </c>
       <c r="F1979" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="1980" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41103,7 +41103,7 @@
         <v>31</v>
       </c>
       <c r="F1984" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="1985" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41123,7 +41123,7 @@
         <v>31</v>
       </c>
       <c r="F1985" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="1986" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41203,7 +41203,7 @@
         <v>7</v>
       </c>
       <c r="F1989" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="1990" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41263,7 +41263,7 @@
         <v>18</v>
       </c>
       <c r="F1992" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="1993" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41303,7 +41303,7 @@
         <v>22</v>
       </c>
       <c r="F1994" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="1995" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -41443,7 +41443,7 @@
         <v>31</v>
       </c>
       <c r="F2001" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2002" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41523,7 +41523,7 @@
         <v>7</v>
       </c>
       <c r="F2005" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2006" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41583,7 +41583,7 @@
         <v>18</v>
       </c>
       <c r="F2008" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2009" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41743,7 +41743,7 @@
         <v>31</v>
       </c>
       <c r="F2016" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2017" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41763,7 +41763,7 @@
         <v>31</v>
       </c>
       <c r="F2017" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2018" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41843,7 +41843,7 @@
         <v>7</v>
       </c>
       <c r="F2021" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2022" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41903,7 +41903,7 @@
         <v>18</v>
       </c>
       <c r="F2024" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2025" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -41943,7 +41943,7 @@
         <v>22</v>
       </c>
       <c r="F2026" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2027" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -42083,7 +42083,7 @@
         <v>31</v>
       </c>
       <c r="F2033" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2034" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42163,7 +42163,7 @@
         <v>7</v>
       </c>
       <c r="F2037" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2038" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42203,7 +42203,7 @@
         <v>18</v>
       </c>
       <c r="F2039" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2040" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42223,7 +42223,7 @@
         <v>18</v>
       </c>
       <c r="F2040" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2041" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42403,7 +42403,7 @@
         <v>31</v>
       </c>
       <c r="F2049" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2050" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42483,7 +42483,7 @@
         <v>7</v>
       </c>
       <c r="F2053" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2054" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42523,7 +42523,7 @@
         <v>18</v>
       </c>
       <c r="F2055" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2056" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42543,7 +42543,7 @@
         <v>18</v>
       </c>
       <c r="F2056" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2057" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42603,7 +42603,7 @@
         <v>22</v>
       </c>
       <c r="F2059" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2060" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42723,7 +42723,7 @@
         <v>31</v>
       </c>
       <c r="F2065" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2066" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42803,7 +42803,7 @@
         <v>7</v>
       </c>
       <c r="F2069" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2070" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42843,7 +42843,7 @@
         <v>18</v>
       </c>
       <c r="F2071" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2072" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42863,7 +42863,7 @@
         <v>18</v>
       </c>
       <c r="F2072" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2073" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -42903,7 +42903,7 @@
         <v>22</v>
       </c>
       <c r="F2074" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2075" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -42963,7 +42963,7 @@
         <v>31</v>
       </c>
       <c r="F2077" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2078" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -43023,7 +43023,7 @@
         <v>31</v>
       </c>
       <c r="F2080" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2081" spans="1:6" ht="30" x14ac:dyDescent="0.2">
@@ -43043,7 +43043,7 @@
         <v>31</v>
       </c>
       <c r="F2081" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2082" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43123,7 +43123,7 @@
         <v>7</v>
       </c>
       <c r="F2085" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2086" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43163,7 +43163,7 @@
         <v>18</v>
       </c>
       <c r="F2087" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2088" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43183,7 +43183,7 @@
         <v>18</v>
       </c>
       <c r="F2088" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2089" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43223,7 +43223,7 @@
         <v>22</v>
       </c>
       <c r="F2090" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2091" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -43323,7 +43323,7 @@
         <v>31</v>
       </c>
       <c r="F2095" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2096" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -43363,7 +43363,7 @@
         <v>31</v>
       </c>
       <c r="F2097" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2098" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43443,7 +43443,7 @@
         <v>7</v>
       </c>
       <c r="F2101" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2102" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43463,7 +43463,7 @@
         <v>7</v>
       </c>
       <c r="F2102" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2103" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43483,7 +43483,7 @@
         <v>18</v>
       </c>
       <c r="F2103" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2104" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43503,7 +43503,7 @@
         <v>18</v>
       </c>
       <c r="F2104" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2105" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43543,7 +43543,7 @@
         <v>22</v>
       </c>
       <c r="F2106" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2107" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -43563,7 +43563,7 @@
         <v>22</v>
       </c>
       <c r="F2107" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2108" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43683,7 +43683,7 @@
         <v>31</v>
       </c>
       <c r="F2113" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2114" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43783,7 +43783,7 @@
         <v>7</v>
       </c>
       <c r="F2118" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2119" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43823,7 +43823,7 @@
         <v>18</v>
       </c>
       <c r="F2120" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2121" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -43863,7 +43863,7 @@
         <v>22</v>
       </c>
       <c r="F2122" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2123" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -44003,7 +44003,7 @@
         <v>31</v>
       </c>
       <c r="F2129" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2130" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44083,7 +44083,7 @@
         <v>7</v>
       </c>
       <c r="F2133" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="2134" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44183,7 +44183,7 @@
         <v>22</v>
       </c>
       <c r="F2138" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2139" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -44303,7 +44303,7 @@
         <v>31</v>
       </c>
       <c r="F2144" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2145" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44323,7 +44323,7 @@
         <v>31</v>
       </c>
       <c r="F2145" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2146" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44403,7 +44403,7 @@
         <v>7</v>
       </c>
       <c r="F2149" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2150" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44443,7 +44443,7 @@
         <v>18</v>
       </c>
       <c r="F2151" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2152" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44483,7 +44483,7 @@
         <v>22</v>
       </c>
       <c r="F2153" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2154" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44503,7 +44503,7 @@
         <v>22</v>
       </c>
       <c r="F2154" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2155" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -44523,7 +44523,7 @@
         <v>22</v>
       </c>
       <c r="F2155" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2156" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44543,7 +44543,7 @@
         <v>22</v>
       </c>
       <c r="F2156" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2157" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44623,7 +44623,7 @@
         <v>31</v>
       </c>
       <c r="F2160" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2161" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44643,7 +44643,7 @@
         <v>31</v>
       </c>
       <c r="F2161" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2162" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44723,7 +44723,7 @@
         <v>7</v>
       </c>
       <c r="F2165" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2166" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44763,7 +44763,7 @@
         <v>18</v>
       </c>
       <c r="F2167" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2168" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44823,7 +44823,7 @@
         <v>22</v>
       </c>
       <c r="F2170" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2171" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -44843,7 +44843,7 @@
         <v>22</v>
       </c>
       <c r="F2171" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2172" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44943,7 +44943,7 @@
         <v>31</v>
       </c>
       <c r="F2176" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2177" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -44963,7 +44963,7 @@
         <v>31</v>
       </c>
       <c r="F2177" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2178" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45043,7 +45043,7 @@
         <v>7</v>
       </c>
       <c r="F2181" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2182" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45083,7 +45083,7 @@
         <v>18</v>
       </c>
       <c r="F2183" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2184" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45103,7 +45103,7 @@
         <v>18</v>
       </c>
       <c r="F2184" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2185" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45143,7 +45143,7 @@
         <v>22</v>
       </c>
       <c r="F2186" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2187" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -45183,7 +45183,7 @@
         <v>22</v>
       </c>
       <c r="F2188" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2189" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45283,7 +45283,7 @@
         <v>31</v>
       </c>
       <c r="F2193" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2194" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45363,7 +45363,7 @@
         <v>7</v>
       </c>
       <c r="F2197" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2198" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45403,7 +45403,7 @@
         <v>18</v>
       </c>
       <c r="F2199" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2200" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45423,7 +45423,7 @@
         <v>18</v>
       </c>
       <c r="F2200" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2201" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45463,7 +45463,7 @@
         <v>22</v>
       </c>
       <c r="F2202" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2203" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -45583,7 +45583,7 @@
         <v>31</v>
       </c>
       <c r="F2208" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2209" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45603,7 +45603,7 @@
         <v>31</v>
       </c>
       <c r="F2209" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2210" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45623,7 +45623,7 @@
         <v>7</v>
       </c>
       <c r="F2210" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2211" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45683,7 +45683,7 @@
         <v>7</v>
       </c>
       <c r="F2213" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2214" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45703,7 +45703,7 @@
         <v>7</v>
       </c>
       <c r="F2214" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2215" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45743,7 +45743,7 @@
         <v>18</v>
       </c>
       <c r="F2216" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2217" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45783,7 +45783,7 @@
         <v>22</v>
       </c>
       <c r="F2218" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="2219" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -45803,7 +45803,7 @@
         <v>22</v>
       </c>
       <c r="F2219" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2220" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45823,7 +45823,7 @@
         <v>22</v>
       </c>
       <c r="F2220" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2221" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45903,7 +45903,7 @@
         <v>31</v>
       </c>
       <c r="F2224" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2225" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -45923,7 +45923,7 @@
         <v>31</v>
       </c>
       <c r="F2225" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2226" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46003,7 +46003,7 @@
         <v>7</v>
       </c>
       <c r="F2229" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2230" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46043,7 +46043,7 @@
         <v>18</v>
       </c>
       <c r="F2231" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2232" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46063,7 +46063,7 @@
         <v>18</v>
       </c>
       <c r="F2232" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2233" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46103,7 +46103,7 @@
         <v>22</v>
       </c>
       <c r="F2234" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2235" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -46123,7 +46123,7 @@
         <v>22</v>
       </c>
       <c r="F2235" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2236" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46223,7 +46223,7 @@
         <v>31</v>
       </c>
       <c r="F2240" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2241" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46243,7 +46243,7 @@
         <v>31</v>
       </c>
       <c r="F2241" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2242" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46303,7 +46303,7 @@
         <v>7</v>
       </c>
       <c r="F2244" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="2245" spans="1:6" ht="45" x14ac:dyDescent="0.2">
@@ -46323,7 +46323,7 @@
         <v>7</v>
       </c>
       <c r="F2245" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2246" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46383,7 +46383,7 @@
         <v>18</v>
       </c>
       <c r="F2248" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2249" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46423,7 +46423,7 @@
         <v>22</v>
       </c>
       <c r="F2250" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2251" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -46543,7 +46543,7 @@
         <v>31</v>
       </c>
       <c r="F2256" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2257" spans="1:6" ht="30" x14ac:dyDescent="0.2">
@@ -46563,7 +46563,7 @@
         <v>31</v>
       </c>
       <c r="F2257" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2258" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46643,7 +46643,7 @@
         <v>7</v>
       </c>
       <c r="F2261" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2262" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46683,7 +46683,7 @@
         <v>18</v>
       </c>
       <c r="F2263" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2264" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46703,7 +46703,7 @@
         <v>18</v>
       </c>
       <c r="F2264" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2265" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46743,7 +46743,7 @@
         <v>22</v>
       </c>
       <c r="F2266" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2267" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -46863,7 +46863,7 @@
         <v>31</v>
       </c>
       <c r="F2272" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2273" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46883,7 +46883,7 @@
         <v>31</v>
       </c>
       <c r="F2273" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2274" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -46963,7 +46963,7 @@
         <v>7</v>
       </c>
       <c r="F2277" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2278" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47003,7 +47003,7 @@
         <v>18</v>
       </c>
       <c r="F2279" s="6" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2280" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47023,7 +47023,7 @@
         <v>18</v>
       </c>
       <c r="F2280" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2281" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47063,7 +47063,7 @@
         <v>22</v>
       </c>
       <c r="F2282" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2283" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -47083,7 +47083,7 @@
         <v>22</v>
       </c>
       <c r="F2283" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="2284" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47103,7 +47103,7 @@
         <v>22</v>
       </c>
       <c r="F2284" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2285" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47183,7 +47183,7 @@
         <v>31</v>
       </c>
       <c r="F2288" s="6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2289" spans="1:6" ht="30" x14ac:dyDescent="0.2">
@@ -47203,7 +47203,7 @@
         <v>31</v>
       </c>
       <c r="F2289" s="6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2290" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47283,7 +47283,7 @@
         <v>7</v>
       </c>
       <c r="F2293" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2294" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47383,7 +47383,7 @@
         <v>22</v>
       </c>
       <c r="F2298" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2299" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -47483,7 +47483,7 @@
         <v>31</v>
       </c>
       <c r="F2303" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2304" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -47503,7 +47503,7 @@
         <v>31</v>
       </c>
       <c r="F2304" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2305" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47523,7 +47523,7 @@
         <v>31</v>
       </c>
       <c r="F2305" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2306" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47603,7 +47603,7 @@
         <v>7</v>
       </c>
       <c r="F2309" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2310" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47643,7 +47643,7 @@
         <v>18</v>
       </c>
       <c r="F2311" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2312" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47683,7 +47683,7 @@
         <v>22</v>
       </c>
       <c r="F2313" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2314" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47723,7 +47723,7 @@
         <v>22</v>
       </c>
       <c r="F2315" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2316" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47743,7 +47743,7 @@
         <v>22</v>
       </c>
       <c r="F2316" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2317" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47803,7 +47803,7 @@
         <v>31</v>
       </c>
       <c r="F2319" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2320" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -47823,7 +47823,7 @@
         <v>31</v>
       </c>
       <c r="F2320" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2321" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47843,7 +47843,7 @@
         <v>31</v>
       </c>
       <c r="F2321" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2322" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47863,7 +47863,7 @@
         <v>7</v>
       </c>
       <c r="F2322" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="2323" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47903,7 +47903,7 @@
         <v>7</v>
       </c>
       <c r="F2324" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2325" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47923,7 +47923,7 @@
         <v>7</v>
       </c>
       <c r="F2325" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2326" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47963,7 +47963,7 @@
         <v>18</v>
       </c>
       <c r="F2327" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2328" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -47983,7 +47983,7 @@
         <v>18</v>
       </c>
       <c r="F2328" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2329" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48043,7 +48043,7 @@
         <v>22</v>
       </c>
       <c r="F2331" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2332" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48063,7 +48063,7 @@
         <v>22</v>
       </c>
       <c r="F2332" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2333" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48103,7 +48103,7 @@
         <v>31</v>
       </c>
       <c r="F2334" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2335" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -48123,7 +48123,7 @@
         <v>31</v>
       </c>
       <c r="F2335" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2336" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -48143,7 +48143,7 @@
         <v>31</v>
       </c>
       <c r="F2336" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2337" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48163,7 +48163,7 @@
         <v>31</v>
       </c>
       <c r="F2337" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2338" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48243,7 +48243,7 @@
         <v>7</v>
       </c>
       <c r="F2341" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="2342" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48283,7 +48283,7 @@
         <v>18</v>
       </c>
       <c r="F2343" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2344" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48303,7 +48303,7 @@
         <v>18</v>
       </c>
       <c r="F2344" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2345" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48463,7 +48463,7 @@
         <v>31</v>
       </c>
       <c r="F2352" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2353" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48483,7 +48483,7 @@
         <v>31</v>
       </c>
       <c r="F2353" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2354" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48563,7 +48563,7 @@
         <v>7</v>
       </c>
       <c r="F2357" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2358" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48603,7 +48603,7 @@
         <v>18</v>
       </c>
       <c r="F2359" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2360" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48663,7 +48663,7 @@
         <v>22</v>
       </c>
       <c r="F2362" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2363" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -48803,7 +48803,7 @@
         <v>31</v>
       </c>
       <c r="F2369" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="2370" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48883,7 +48883,7 @@
         <v>7</v>
       </c>
       <c r="F2373" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2374" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48923,7 +48923,7 @@
         <v>18</v>
       </c>
       <c r="F2375" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2376" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48943,7 +48943,7 @@
         <v>18</v>
       </c>
       <c r="F2376" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2377" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48963,7 +48963,7 @@
         <v>22</v>
       </c>
       <c r="F2377" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="2378" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -48983,7 +48983,7 @@
         <v>22</v>
       </c>
       <c r="F2378" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2379" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -49043,7 +49043,7 @@
         <v>31</v>
       </c>
       <c r="F2381" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2382" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -49103,7 +49103,7 @@
         <v>31</v>
       </c>
       <c r="F2384" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2385" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49123,7 +49123,7 @@
         <v>31</v>
       </c>
       <c r="F2385" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2386" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49223,7 +49223,7 @@
         <v>7</v>
       </c>
       <c r="F2390" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2391" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49263,7 +49263,7 @@
         <v>18</v>
       </c>
       <c r="F2392" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2393" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49283,7 +49283,7 @@
         <v>22</v>
       </c>
       <c r="F2393" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2394" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49323,7 +49323,7 @@
         <v>22</v>
       </c>
       <c r="F2395" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2396" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49343,7 +49343,7 @@
         <v>22</v>
       </c>
       <c r="F2396" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2397" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -49443,7 +49443,7 @@
         <v>31</v>
       </c>
       <c r="F2401" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>